<commit_message>
modificaions génération chapitres avant réécriture complète de la logique de traitement par Deepseek
</commit_message>
<xml_diff>
--- a/tools_xlsx/cours.xlsx
+++ b/tools_xlsx/cours.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LYCEE ACAJOU 2\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\electron\coursInteractifs\tools_xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="43">
   <si>
     <t>type</t>
   </si>
@@ -712,9 +712,6 @@
       <c r="I6" t="s">
         <v>19</v>
       </c>
-      <c r="J6" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="7" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">

</xml_diff>

<commit_message>
feat: finalisation du générateur de chapitres et du système de suivi
- Correction du calcul des pénalités (max 2×points)
- Uniformisation des IDs de feedback
- Ajout du mode examen avec validation globale
- Système de suivi des tentatives pour questions auto-corrigées
- Calcul de note avec formule N×(1+p)/2
- Affichage des statistiques de progression
- Correction des QCM multiples et sélections
- Gestion des réponses courtes et ouvertes
- Amélioration du dashboard professeur
- Ajout de la classe hidden pour le bouton global
</commit_message>
<xml_diff>
--- a/tools_xlsx/cours.xlsx
+++ b/tools_xlsx/cours.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="41">
   <si>
     <t>type</t>
   </si>
@@ -74,9 +74,6 @@
 L'annexe 1 présente un rappel sur les dictionnaires en langage Python (voir en bas de page, avec quelques exercices d'échauffement si nécessaire) .</t>
   </si>
   <si>
-    <t>contenu (format markdow Capytale)</t>
-  </si>
-  <si>
     <t>qcm</t>
   </si>
   <si>
@@ -98,22 +95,13 @@
     <t>## Quelle est la couleur du cheval blanc d'henri 4</t>
   </si>
   <si>
-    <t>type réponse</t>
-  </si>
-  <si>
     <t>validation</t>
   </si>
   <si>
-    <t>type correction</t>
-  </si>
-  <si>
     <t>auto</t>
   </si>
   <si>
     <t>choix</t>
-  </si>
-  <si>
-    <t>choix correct(s)</t>
   </si>
   <si>
     <t xml:space="preserve">bleu
@@ -128,15 +116,6 @@
     <t>points</t>
   </si>
   <si>
-    <t>règle</t>
-  </si>
-  <si>
-    <t>obligatoire</t>
-  </si>
-  <si>
-    <t>facultatif</t>
-  </si>
-  <si>
     <t>## Quelle est la couleur du cheval blanc d'henri 4, fais moi une dissertation sur ce thème</t>
   </si>
   <si>
@@ -151,9 +130,6 @@
   <si>
     <t>blanche
 blanc</t>
-  </si>
-  <si>
-    <t>ordre choix</t>
   </si>
   <si>
     <t>aleatoire</t>
@@ -172,9 +148,6 @@
 </t>
   </si>
   <si>
-    <t>1;3</t>
-  </si>
-  <si>
     <t>indication</t>
   </si>
   <si>
@@ -197,6 +170,27 @@
   </si>
   <si>
     <t>Un nombre entier et c'est pas 5</t>
+  </si>
+  <si>
+    <t>contenu</t>
+  </si>
+  <si>
+    <t>correction</t>
+  </si>
+  <si>
+    <t>ordre_choix</t>
+  </si>
+  <si>
+    <t>choix_corrects</t>
+  </si>
+  <si>
+    <t>regle</t>
+  </si>
+  <si>
+    <t>texte(10)</t>
+  </si>
+  <si>
+    <t>2;4</t>
   </si>
 </sst>
 </file>
@@ -517,46 +511,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="54" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="79.81640625" customWidth="1"/>
-    <col min="3" max="4" width="14.08984375" customWidth="1"/>
+    <col min="3" max="3" width="14.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H1" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="I1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -564,31 +555,28 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="54" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -596,217 +584,196 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="96.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="1">
+        <v>4</v>
+      </c>
+      <c r="I8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4">
+      <c r="H9">
         <v>2</v>
       </c>
-      <c r="J4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7">
-        <v>2</v>
-      </c>
-      <c r="G7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" t="s">
-        <v>19</v>
-      </c>
-      <c r="I7" s="1" t="s">
+      <c r="I9" t="s">
         <v>28</v>
-      </c>
-      <c r="J7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8">
-        <v>3</v>
-      </c>
-      <c r="G8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I8" s="1">
-        <v>4</v>
-      </c>
-      <c r="J8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9">
-        <v>2</v>
-      </c>
-      <c r="J9" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: version Correction modal 3 onglets (tous, auto-corrigé et à corriger)
</commit_message>
<xml_diff>
--- a/tools_xlsx/cours.xlsx
+++ b/tools_xlsx/cours.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
   <si>
     <t>type</t>
   </si>
@@ -190,7 +190,11 @@
     <t>texte(10)</t>
   </si>
   <si>
-    <t>2;4</t>
+    <t>blanc
+noire</t>
+  </si>
+  <si>
+    <t>blanc</t>
   </si>
 </sst>
 </file>
@@ -627,8 +631,8 @@
       <c r="G4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H4">
-        <v>2</v>
+      <c r="H4" t="s">
+        <v>41</v>
       </c>
       <c r="I4" t="s">
         <v>28</v>
@@ -656,7 +660,7 @@
       <c r="G5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>40</v>
       </c>
       <c r="I5" t="s">
@@ -769,8 +773,8 @@
       <c r="G9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H9">
-        <v>2</v>
+      <c r="H9" t="s">
+        <v>41</v>
       </c>
       <c r="I9" t="s">
         <v>28</v>

</xml_diff>